<commit_message>
Update seminars.xlsx and upcoming.xlsx
</commit_message>
<xml_diff>
--- a/data/seminars.xlsx
+++ b/data/seminars.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sigrid\Documents\BES\work\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sigrid\Documents\BES\BES_new\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="4080" windowHeight="11370"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11715"/>
   </bookViews>
   <sheets>
     <sheet name="Conferences" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="112">
   <si>
     <t>date</t>
   </si>
@@ -316,9 +316,6 @@
     <t>Collaborate to innovate: iptacopan and RWE in PNH treatment</t>
   </si>
   <si>
-    <t>4_Fermont.pdf</t>
-  </si>
-  <si>
     <t>retention policy</t>
   </si>
   <si>
@@ -347,6 +344,30 @@
   </si>
   <si>
     <t>13.06.2024</t>
+  </si>
+  <si>
+    <t>16.09.2026</t>
+  </si>
+  <si>
+    <t>Zooming in on Feasibility Assessments and Data Quality</t>
+  </si>
+  <si>
+    <t>Sigrid Behr</t>
+  </si>
+  <si>
+    <t>Introduction</t>
+  </si>
+  <si>
+    <t>Christian Selinger</t>
+  </si>
+  <si>
+    <t>Malaria routine surveillance data for population health: use cases and challenges</t>
+  </si>
+  <si>
+    <t>Jocelyn Buisker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementing a risk-based data quality framework for a post-authorization safety study </t>
   </si>
 </sst>
 </file>
@@ -498,7 +519,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="9525" cy="9525"/>
@@ -532,7 +553,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="9525" cy="9525"/>
@@ -832,7 +853,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L655"/>
+  <dimension ref="A1:L658"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.85546875" style="8" customWidth="1"/>
@@ -884,7 +905,7 @@
         <v>8</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="28.5" x14ac:dyDescent="0.2">
@@ -892,7 +913,7 @@
         <v>104</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>81</v>
+        <v>105</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -901,27 +922,22 @@
         <v>1</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>82</v>
+        <v>106</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>83</v>
+        <v>11</v>
       </c>
       <c r="I2" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="L2" s="7" t="s">
-        <v>96</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="J2" s="2"/>
     </row>
     <row r="3" spans="1:12" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A3" s="17" t="s">
         <v>104</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>81</v>
+        <v>105</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -930,27 +946,22 @@
         <v>2</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>14</v>
+        <v>61</v>
       </c>
       <c r="I3" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="L3" s="7" t="s">
-        <v>96</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="J3" s="2"/>
     </row>
     <row r="4" spans="1:12" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A4" s="17" t="s">
         <v>104</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>81</v>
+        <v>105</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
@@ -959,24 +970,19 @@
         <v>3</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>89</v>
+        <v>110</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="L4" s="7" t="s">
-        <v>96</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="J4" s="2"/>
     </row>
     <row r="5" spans="1:12" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B5" s="16" t="s">
         <v>81</v>
@@ -985,27 +991,27 @@
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>11</v>
+        <v>83</v>
       </c>
       <c r="I5" s="13" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A6" s="17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B6" s="16" t="s">
         <v>81</v>
@@ -1014,27 +1020,27 @@
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
       <c r="F6" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>59</v>
+        <v>86</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>83</v>
+        <v>14</v>
       </c>
       <c r="I6" s="13" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A7" s="17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B7" s="16" t="s">
         <v>81</v>
@@ -1043,113 +1049,111 @@
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
       <c r="F7" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="J7" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A8" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="L7" s="7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7">
-        <v>1</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>27</v>
-      </c>
+      <c r="B8" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="1">
+        <v>4</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I8" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="J8" s="2"/>
       <c r="L8" s="7" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7">
-        <v>2</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I9" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="J9" s="7" t="s">
-        <v>26</v>
+    <row r="9" spans="1:12" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A9" s="17" t="s">
+        <v>103</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="1">
+        <v>5</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="I9" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>98</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7">
-        <v>3</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="I10" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J10" s="7" t="s">
-        <v>25</v>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A10" s="17" t="s">
+        <v>103</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="1">
+        <v>6</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="I10" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>102</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="18" t="s">
         <v>28</v>
       </c>
       <c r="B11" s="3" t="s">
@@ -1159,109 +1163,109 @@
       <c r="D11" s="7"/>
       <c r="E11" s="7"/>
       <c r="F11" s="7">
+        <v>1</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="3"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7">
+        <v>2</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="L12" s="7" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="3"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7">
+        <v>3</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="3"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7">
         <v>4</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G14" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H14" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="I11" s="7" t="s">
+      <c r="I14" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="J11" s="7" t="s">
+      <c r="J14" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="L11" s="7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="3">
-        <v>1</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I12" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="J12" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="L12" s="7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="3">
-        <v>2</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="J13" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="L13" s="7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="3">
-        <v>3</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="J14" s="15" t="s">
-        <v>51</v>
-      </c>
       <c r="L14" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -1275,25 +1279,25 @@
       <c r="D15" s="11"/>
       <c r="E15" s="11"/>
       <c r="F15" s="3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="J15" s="15" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
         <v>29</v>
       </c>
@@ -1304,22 +1308,22 @@
       <c r="D16" s="11"/>
       <c r="E16" s="11"/>
       <c r="F16" s="3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="J16" s="15" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
@@ -1333,22 +1337,22 @@
       <c r="D17" s="11"/>
       <c r="E17" s="11"/>
       <c r="F17" s="3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="J17" s="15" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="L17" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
@@ -1362,94 +1366,94 @@
       <c r="D18" s="11"/>
       <c r="E18" s="11"/>
       <c r="F18" s="3">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="J18" s="15" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="C19" s="11"/>
       <c r="D19" s="11"/>
       <c r="E19" s="11"/>
       <c r="F19" s="3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>58</v>
+        <v>35</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="J19" s="15" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="L19" s="7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="C20" s="11"/>
       <c r="D20" s="11"/>
       <c r="E20" s="11"/>
       <c r="F20" s="3">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="J20" s="15" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" ht="42.75" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="C21" s="11"/>
       <c r="D21" s="11"/>
       <c r="E21" s="11"/>
       <c r="F21" s="3">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G21" s="4" t="s">
         <v>37</v>
@@ -1458,21 +1462,21 @@
         <v>13</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="J21" s="15" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="L21" s="7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" ht="42.75" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="C22" s="11"/>
       <c r="D22" s="11"/>
@@ -1481,27 +1485,27 @@
         <v>1</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="J22" s="15" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" ht="42.75" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="C23" s="11"/>
       <c r="D23" s="11"/>
@@ -1510,27 +1514,27 @@
         <v>2</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="J23" s="15" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="L23" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:12" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A24" s="17" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="C24" s="11"/>
       <c r="D24" s="11"/>
@@ -1539,56 +1543,107 @@
         <v>3</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>74</v>
+        <v>37</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>61</v>
+        <v>13</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="J24" s="15" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="L24" s="7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A25" s="9"/>
-      <c r="B25" s="12"/>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="42.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>69</v>
+      </c>
       <c r="C25" s="11"/>
       <c r="D25" s="11"/>
       <c r="E25" s="11"/>
-      <c r="F25" s="3"/>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="1"/>
-      <c r="J25" s="15"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A26" s="9"/>
-      <c r="B26" s="12"/>
+      <c r="F25" s="3">
+        <v>1</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="J25" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="L25" s="7" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="42.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>69</v>
+      </c>
       <c r="C26" s="11"/>
       <c r="D26" s="11"/>
       <c r="E26" s="11"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="1"/>
-      <c r="J26" s="15"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A27" s="9"/>
-      <c r="B27" s="12"/>
+      <c r="F26" s="3">
+        <v>2</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="J26" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="L26" s="7" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="42.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>69</v>
+      </c>
       <c r="C27" s="11"/>
       <c r="D27" s="11"/>
       <c r="E27" s="11"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="1"/>
-      <c r="J27" s="15"/>
+      <c r="F27" s="3">
+        <v>3</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="J27" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="L27" s="7" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="9"/>
@@ -2611,40 +2666,40 @@
       <c r="J112" s="15"/>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A113" s="10"/>
-      <c r="B113" s="6"/>
-      <c r="C113" s="4"/>
-      <c r="D113" s="4"/>
-      <c r="E113" s="4"/>
-      <c r="F113" s="2"/>
+      <c r="A113" s="9"/>
+      <c r="B113" s="12"/>
+      <c r="C113" s="11"/>
+      <c r="D113" s="11"/>
+      <c r="E113" s="11"/>
+      <c r="F113" s="3"/>
       <c r="G113" s="4"/>
       <c r="H113" s="4"/>
-      <c r="I113" s="13"/>
-      <c r="J113" s="2"/>
+      <c r="I113" s="1"/>
+      <c r="J113" s="15"/>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A114" s="10"/>
-      <c r="B114" s="6"/>
-      <c r="C114" s="4"/>
-      <c r="D114" s="4"/>
-      <c r="E114" s="4"/>
-      <c r="F114" s="2"/>
+      <c r="A114" s="9"/>
+      <c r="B114" s="12"/>
+      <c r="C114" s="11"/>
+      <c r="D114" s="11"/>
+      <c r="E114" s="11"/>
+      <c r="F114" s="3"/>
       <c r="G114" s="4"/>
       <c r="H114" s="4"/>
-      <c r="I114" s="13"/>
-      <c r="J114" s="2"/>
+      <c r="I114" s="1"/>
+      <c r="J114" s="15"/>
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A115" s="10"/>
-      <c r="B115" s="6"/>
-      <c r="C115" s="4"/>
-      <c r="D115" s="4"/>
-      <c r="E115" s="4"/>
-      <c r="F115" s="2"/>
+      <c r="A115" s="9"/>
+      <c r="B115" s="12"/>
+      <c r="C115" s="11"/>
+      <c r="D115" s="11"/>
+      <c r="E115" s="11"/>
+      <c r="F115" s="3"/>
       <c r="G115" s="4"/>
       <c r="H115" s="4"/>
-      <c r="I115" s="13"/>
-      <c r="J115" s="2"/>
+      <c r="I115" s="1"/>
+      <c r="J115" s="15"/>
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A116" s="10"/>
@@ -9126,6 +9181,42 @@
       <c r="I655" s="13"/>
       <c r="J655" s="2"/>
     </row>
+    <row r="656" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A656" s="10"/>
+      <c r="B656" s="6"/>
+      <c r="C656" s="4"/>
+      <c r="D656" s="4"/>
+      <c r="E656" s="4"/>
+      <c r="F656" s="2"/>
+      <c r="G656" s="4"/>
+      <c r="H656" s="4"/>
+      <c r="I656" s="13"/>
+      <c r="J656" s="2"/>
+    </row>
+    <row r="657" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A657" s="10"/>
+      <c r="B657" s="6"/>
+      <c r="C657" s="4"/>
+      <c r="D657" s="4"/>
+      <c r="E657" s="4"/>
+      <c r="F657" s="2"/>
+      <c r="G657" s="4"/>
+      <c r="H657" s="4"/>
+      <c r="I657" s="13"/>
+      <c r="J657" s="2"/>
+    </row>
+    <row r="658" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A658" s="10"/>
+      <c r="B658" s="6"/>
+      <c r="C658" s="4"/>
+      <c r="D658" s="4"/>
+      <c r="E658" s="4"/>
+      <c r="F658" s="2"/>
+      <c r="G658" s="4"/>
+      <c r="H658" s="4"/>
+      <c r="I658" s="13"/>
+      <c r="J658" s="2"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>